<commit_message>
docs(agency): mark TC-AGENCY-020 and TC-AGENCY-049 as Rejected
Operator ruling 2026-08-20: both are confirmed system behaviour, not
defects. Sync Markdown Review/Automation status and summary table to
match the Excel edit; Expected Result text left unchanged.
</commit_message>
<xml_diff>
--- a/platform_core_data/modules/agency/test_design/TestCases_Agency.xlsx
+++ b/platform_core_data/modules/agency/test_design/TestCases_Agency.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="10980"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="Agency" sheetId="1" r:id="rId1"/>
@@ -1905,7 +1905,7 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -3391,10 +3391,10 @@
         <v>169</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" ht="60" spans="1:12">
@@ -4454,10 +4454,10 @@
         <v>368</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" ht="240" spans="1:12">

</xml_diff>